<commit_message>
validaciones de instrucciones del excel
</commit_message>
<xml_diff>
--- a/OneDrive - Aris-Mining/Escritorio/proyecto/frontend/public/plantilla-operarios.xlsx
+++ b/OneDrive - Aris-Mining/Escritorio/proyecto/frontend/public/plantilla-operarios.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://arismining-my.sharepoint.com/personal/mariana_penagos_aris-mining_co/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mariana.penagos\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="8_{390D9ADA-A695-4C5C-9663-F0C271075452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5637C532-8961-49D5-B5AC-F379F516F815}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8298552-1481-4916-8358-B6DC27804BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{903069D3-1599-4C3F-9137-A790A31C4727}"/>
   </bookViews>
@@ -36,18 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t xml:space="preserve"> Puesto </t>
   </si>
   <si>
     <t xml:space="preserve"> Departamento </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Sede</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CREACIÓN DE USUARIOS - OPERARIOS </t>
   </si>
   <si>
     <t xml:space="preserve">Primer Nombre </t>
@@ -60,6 +54,15 @@
   </si>
   <si>
     <t xml:space="preserve"> Segundo Apellido </t>
+  </si>
+  <si>
+    <t>CREACIÓN DE USUARIOS - OPERARIOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Codigo Postal </t>
+  </si>
+  <si>
+    <t>Sede</t>
   </si>
 </sst>
 </file>
@@ -142,10 +145,10 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
+      <left style="thin">
         <color indexed="64"/>
-      </right>
+      </left>
+      <right/>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -156,19 +159,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -512,9 +521,8 @@
   <cols>
     <col min="1" max="1" width="13.7265625" customWidth="1"/>
     <col min="2" max="2" width="15.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.90625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.81640625" customWidth="1"/>
@@ -526,380 +534,422 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
-        <v>3</v>
+      <c r="A1" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
-      <c r="G1" s="5"/>
-      <c r="N1" s="3"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="N1" s="2"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
+      <c r="E2" s="5" t="s">
+        <v>0</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" formatCells="0" formatColumns="0" insertColumns="0" insertRows="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Selección no válida" error="Debe seleccionar una opción válida desde la lista desplegable._x000a_No está permitido ingresar texto manualmente." sqref="G3:G39" xr:uid="{1EB79CD0-9DCF-49EE-848B-9C7CB9FF2F7A}">
+  <dataValidations count="2">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Selección no válida" error="Debe seleccionar una opción válida desde la lista desplegable._x000a_No está permitido ingresar texto manualmente." sqref="F3:F39 H3" xr:uid="{1EB79CD0-9DCF-49EE-848B-9C7CB9FF2F7A}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Selección no válida" error="Debe seleccionar una opción válida desde la lista desplegable._x000a_No está permitido ingresar texto manualmente." sqref="G3:G39" xr:uid="{117944FF-2253-4FD3-831E-7C161DBF6AD9}">
       <formula1>"Medellín,Segovia,Marmato,Bogotá,Bucaramanga"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>